<commit_message>
Stage and push all changes
</commit_message>
<xml_diff>
--- a/BANA6420_Gill,Nathanael_Unit4Assignment.xlsx
+++ b/BANA6420_Gill,Nathanael_Unit4Assignment.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calculations" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,7 +17,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="23">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -123,6 +124,17 @@
       <name val="Arial"/>
       <color rgb="FFFFFFFF"/>
       <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -363,7 +375,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -526,6 +538,23 @@
     <xf numFmtId="2" fontId="9" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -15760,4 +15789,1012 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="43" min="1" max="1"/>
+    <col width="16" customWidth="1" style="43" min="2" max="2"/>
+    <col width="16" customWidth="1" style="43" min="3" max="3"/>
+    <col width="24" customWidth="1" style="43" min="4" max="4"/>
+    <col width="24" customWidth="1" style="43" min="5" max="5"/>
+    <col width="24" customWidth="1" style="43" min="6" max="6"/>
+    <col width="24" customWidth="1" style="43" min="7" max="7"/>
+    <col width="24" customWidth="1" style="43" min="8" max="8"/>
+    <col width="24" customWidth="1" style="43" min="9" max="9"/>
+    <col width="24" customWidth="1" style="43" min="10" max="10"/>
+    <col width="24" customWidth="1" style="43" min="11" max="11"/>
+    <col width="24" customWidth="1" style="43" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="60" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B1" s="60" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="C1" s="60" t="inlineStr">
+        <is>
+          <t>Year</t>
+        </is>
+      </c>
+      <c r="D1" s="60" t="inlineStr">
+        <is>
+          <t>Accounts Receivable (USD)</t>
+        </is>
+      </c>
+      <c r="E1" s="60" t="inlineStr">
+        <is>
+          <t>Inventory (USD)</t>
+        </is>
+      </c>
+      <c r="F1" s="60" t="inlineStr">
+        <is>
+          <t>Accounts Payable (USD)</t>
+        </is>
+      </c>
+      <c r="G1" s="60" t="inlineStr">
+        <is>
+          <t>Annual Sales (USD)</t>
+        </is>
+      </c>
+      <c r="H1" s="60" t="inlineStr">
+        <is>
+          <t>Annual COGS (USD)</t>
+        </is>
+      </c>
+      <c r="I1" s="60" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="J1" s="60" t="inlineStr">
+        <is>
+          <t>DI</t>
+        </is>
+      </c>
+      <c r="K1" s="60" t="inlineStr">
+        <is>
+          <t>DAP</t>
+        </is>
+      </c>
+      <c r="L1" s="60" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>3M COMPANY</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D2" s="61">
+        <f>'Data'!C3*1000000</f>
+        <v/>
+      </c>
+      <c r="E2" s="61">
+        <f>'Data'!C4*1000000</f>
+        <v/>
+      </c>
+      <c r="F2" s="61">
+        <f>'Data'!C5*1000000</f>
+        <v/>
+      </c>
+      <c r="G2" s="61">
+        <f>'Data'!C6*1000000</f>
+        <v/>
+      </c>
+      <c r="H2" s="61">
+        <f>'Data'!C7*1000000</f>
+        <v/>
+      </c>
+      <c r="I2" s="62">
+        <f>IFERROR((D2/G2)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J2" s="62">
+        <f>IFERROR((E2/H2)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K2" s="62">
+        <f>IFERROR((F2/H2)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L2" s="62">
+        <f>IFERROR(I2+J2-K2,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>3M COMPANY</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D3" s="61">
+        <f>'Data'!D3*1000000</f>
+        <v/>
+      </c>
+      <c r="E3" s="61">
+        <f>'Data'!D4*1000000</f>
+        <v/>
+      </c>
+      <c r="F3" s="61">
+        <f>'Data'!D5*1000000</f>
+        <v/>
+      </c>
+      <c r="G3" s="61">
+        <f>'Data'!D6*1000000</f>
+        <v/>
+      </c>
+      <c r="H3" s="61">
+        <f>'Data'!D7*1000000</f>
+        <v/>
+      </c>
+      <c r="I3" s="62">
+        <f>IFERROR((D3/G3)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J3" s="62">
+        <f>IFERROR((E3/H3)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K3" s="62">
+        <f>IFERROR((F3/H3)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L3" s="62">
+        <f>IFERROR(I3+J3-K3,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3M COMPANY</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D4" s="61">
+        <f>'Data'!E3*1000000</f>
+        <v/>
+      </c>
+      <c r="E4" s="61">
+        <f>'Data'!E4*1000000</f>
+        <v/>
+      </c>
+      <c r="F4" s="61">
+        <f>'Data'!E5*1000000</f>
+        <v/>
+      </c>
+      <c r="G4" s="61">
+        <f>'Data'!E6*1000000</f>
+        <v/>
+      </c>
+      <c r="H4" s="61">
+        <f>'Data'!E7*1000000</f>
+        <v/>
+      </c>
+      <c r="I4" s="62">
+        <f>IFERROR((D4/G4)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J4" s="62">
+        <f>IFERROR((E4/H4)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K4" s="62">
+        <f>IFERROR((F4/H4)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L4" s="62">
+        <f>IFERROR(I4+J4-K4,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>3M COMPANY</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D5" s="61">
+        <f>'Data'!F3*1000000</f>
+        <v/>
+      </c>
+      <c r="E5" s="61">
+        <f>'Data'!F4*1000000</f>
+        <v/>
+      </c>
+      <c r="F5" s="61">
+        <f>'Data'!F5*1000000</f>
+        <v/>
+      </c>
+      <c r="G5" s="61">
+        <f>'Data'!F6*1000000</f>
+        <v/>
+      </c>
+      <c r="H5" s="61">
+        <f>'Data'!F7*1000000</f>
+        <v/>
+      </c>
+      <c r="I5" s="62">
+        <f>IFERROR((D5/G5)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J5" s="62">
+        <f>IFERROR((E5/H5)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="62">
+        <f>IFERROR((F5/H5)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L5" s="62">
+        <f>IFERROR(I5+J5-K5,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3M COMPANY</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D6" s="61">
+        <f>'Data'!G3*1000000</f>
+        <v/>
+      </c>
+      <c r="E6" s="61">
+        <f>'Data'!G4*1000000</f>
+        <v/>
+      </c>
+      <c r="F6" s="61">
+        <f>'Data'!G5*1000000</f>
+        <v/>
+      </c>
+      <c r="G6" s="61">
+        <f>'Data'!G6*1000000</f>
+        <v/>
+      </c>
+      <c r="H6" s="61">
+        <f>'Data'!G7*1000000</f>
+        <v/>
+      </c>
+      <c r="I6" s="62">
+        <f>IFERROR((D6/G6)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="62">
+        <f>IFERROR((E6/H6)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="62">
+        <f>IFERROR((F6/H6)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="62">
+        <f>IFERROR(I6+J6-K6,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3M COMPANY</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D7" s="61">
+        <f>'Data'!H3*1000000</f>
+        <v/>
+      </c>
+      <c r="E7" s="61">
+        <f>'Data'!H4*1000000</f>
+        <v/>
+      </c>
+      <c r="F7" s="61">
+        <f>'Data'!H5*1000000</f>
+        <v/>
+      </c>
+      <c r="G7" s="61">
+        <f>'Data'!H6*1000000</f>
+        <v/>
+      </c>
+      <c r="H7" s="61">
+        <f>'Data'!H7*1000000</f>
+        <v/>
+      </c>
+      <c r="I7" s="62">
+        <f>IFERROR((D7/G7)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="62">
+        <f>IFERROR((E7/H7)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="62">
+        <f>IFERROR((F7/H7)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="62">
+        <f>IFERROR(I7+J7-K7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>PROCTER &amp; GAMBLE CO</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D8" s="61">
+        <f>'Data'!C14*1000000</f>
+        <v/>
+      </c>
+      <c r="E8" s="61">
+        <f>'Data'!C15*1000000</f>
+        <v/>
+      </c>
+      <c r="F8" s="61">
+        <f>'Data'!C16*1000000</f>
+        <v/>
+      </c>
+      <c r="G8" s="61">
+        <f>'Data'!C17*1000000</f>
+        <v/>
+      </c>
+      <c r="H8" s="61">
+        <f>'Data'!C18*1000000</f>
+        <v/>
+      </c>
+      <c r="I8" s="62">
+        <f>IFERROR((D8/G8)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="62">
+        <f>IFERROR((E8/H8)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="62">
+        <f>IFERROR((F8/H8)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="62">
+        <f>IFERROR(I8+J8-K8,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>PROCTER &amp; GAMBLE CO</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D9" s="61">
+        <f>'Data'!D14*1000000</f>
+        <v/>
+      </c>
+      <c r="E9" s="61">
+        <f>'Data'!D15*1000000</f>
+        <v/>
+      </c>
+      <c r="F9" s="61">
+        <f>'Data'!D16*1000000</f>
+        <v/>
+      </c>
+      <c r="G9" s="61">
+        <f>'Data'!D17*1000000</f>
+        <v/>
+      </c>
+      <c r="H9" s="61">
+        <f>'Data'!D18*1000000</f>
+        <v/>
+      </c>
+      <c r="I9" s="62">
+        <f>IFERROR((D9/G9)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="62">
+        <f>IFERROR((E9/H9)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="62">
+        <f>IFERROR((F9/H9)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="62">
+        <f>IFERROR(I9+J9-K9,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>PROCTER &amp; GAMBLE CO</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D10" s="61">
+        <f>'Data'!E14*1000000</f>
+        <v/>
+      </c>
+      <c r="E10" s="61">
+        <f>'Data'!E15*1000000</f>
+        <v/>
+      </c>
+      <c r="F10" s="61">
+        <f>'Data'!E16*1000000</f>
+        <v/>
+      </c>
+      <c r="G10" s="61">
+        <f>'Data'!E17*1000000</f>
+        <v/>
+      </c>
+      <c r="H10" s="61">
+        <f>'Data'!E18*1000000</f>
+        <v/>
+      </c>
+      <c r="I10" s="62">
+        <f>IFERROR((D10/G10)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="62">
+        <f>IFERROR((E10/H10)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="62">
+        <f>IFERROR((F10/H10)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="62">
+        <f>IFERROR(I10+J10-K10,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>PROCTER &amp; GAMBLE CO</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D11" s="61">
+        <f>'Data'!F14*1000000</f>
+        <v/>
+      </c>
+      <c r="E11" s="61">
+        <f>'Data'!F15*1000000</f>
+        <v/>
+      </c>
+      <c r="F11" s="61">
+        <f>'Data'!F16*1000000</f>
+        <v/>
+      </c>
+      <c r="G11" s="61">
+        <f>'Data'!F17*1000000</f>
+        <v/>
+      </c>
+      <c r="H11" s="61">
+        <f>'Data'!F18*1000000</f>
+        <v/>
+      </c>
+      <c r="I11" s="62">
+        <f>IFERROR((D11/G11)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="62">
+        <f>IFERROR((E11/H11)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="62">
+        <f>IFERROR((F11/H11)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="62">
+        <f>IFERROR(I11+J11-K11,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PROCTER &amp; GAMBLE CO</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D12" s="61">
+        <f>'Data'!G14*1000000</f>
+        <v/>
+      </c>
+      <c r="E12" s="61">
+        <f>'Data'!G15*1000000</f>
+        <v/>
+      </c>
+      <c r="F12" s="61">
+        <f>'Data'!G16*1000000</f>
+        <v/>
+      </c>
+      <c r="G12" s="61">
+        <f>'Data'!G17*1000000</f>
+        <v/>
+      </c>
+      <c r="H12" s="61">
+        <f>'Data'!G18*1000000</f>
+        <v/>
+      </c>
+      <c r="I12" s="62">
+        <f>IFERROR((D12/G12)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="62">
+        <f>IFERROR((E12/H12)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="62">
+        <f>IFERROR((F12/H12)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="62">
+        <f>IFERROR(I12+J12-K12,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PROCTER &amp; GAMBLE CO</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D13" s="61">
+        <f>'Data'!H14*1000000</f>
+        <v/>
+      </c>
+      <c r="E13" s="61">
+        <f>'Data'!H15*1000000</f>
+        <v/>
+      </c>
+      <c r="F13" s="61">
+        <f>'Data'!H16*1000000</f>
+        <v/>
+      </c>
+      <c r="G13" s="61">
+        <f>'Data'!H17*1000000</f>
+        <v/>
+      </c>
+      <c r="H13" s="61">
+        <f>'Data'!H18*1000000</f>
+        <v/>
+      </c>
+      <c r="I13" s="62">
+        <f>IFERROR((D13/G13)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="62">
+        <f>IFERROR((E13/H13)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="62">
+        <f>IFERROR((F13/H13)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="62">
+        <f>IFERROR(I13+J13-K13,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>2016</v>
+      </c>
+      <c r="D14" s="61">
+        <f>'Data'!C25*1000000</f>
+        <v/>
+      </c>
+      <c r="E14" s="61">
+        <f>'Data'!C26*1000000</f>
+        <v/>
+      </c>
+      <c r="F14" s="61">
+        <f>'Data'!C27*1000000</f>
+        <v/>
+      </c>
+      <c r="G14" s="61">
+        <f>'Data'!C28*1000000</f>
+        <v/>
+      </c>
+      <c r="H14" s="61">
+        <f>'Data'!C29*1000000</f>
+        <v/>
+      </c>
+      <c r="I14" s="62">
+        <f>IFERROR((D14/G14)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="62">
+        <f>IFERROR((E14/H14)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="62">
+        <f>IFERROR((F14/H14)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="62">
+        <f>IFERROR(I14+J14-K14,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2017</v>
+      </c>
+      <c r="D15" s="61">
+        <f>'Data'!D25*1000000</f>
+        <v/>
+      </c>
+      <c r="E15" s="61">
+        <f>'Data'!D26*1000000</f>
+        <v/>
+      </c>
+      <c r="F15" s="61">
+        <f>'Data'!D27*1000000</f>
+        <v/>
+      </c>
+      <c r="G15" s="61">
+        <f>'Data'!D28*1000000</f>
+        <v/>
+      </c>
+      <c r="H15" s="61">
+        <f>'Data'!D29*1000000</f>
+        <v/>
+      </c>
+      <c r="I15" s="62">
+        <f>IFERROR((D15/G15)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="62">
+        <f>IFERROR((E15/H15)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="62">
+        <f>IFERROR((F15/H15)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="62">
+        <f>IFERROR(I15+J15-K15,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2018</v>
+      </c>
+      <c r="D16" s="61">
+        <f>'Data'!E25*1000000</f>
+        <v/>
+      </c>
+      <c r="E16" s="61">
+        <f>'Data'!E26*1000000</f>
+        <v/>
+      </c>
+      <c r="F16" s="61">
+        <f>'Data'!E27*1000000</f>
+        <v/>
+      </c>
+      <c r="G16" s="61">
+        <f>'Data'!E28*1000000</f>
+        <v/>
+      </c>
+      <c r="H16" s="61">
+        <f>'Data'!E29*1000000</f>
+        <v/>
+      </c>
+      <c r="I16" s="62">
+        <f>IFERROR((D16/G16)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="62">
+        <f>IFERROR((E16/H16)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="62">
+        <f>IFERROR((F16/H16)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="62">
+        <f>IFERROR(I16+J16-K16,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2019</v>
+      </c>
+      <c r="D17" s="61">
+        <f>'Data'!F25*1000000</f>
+        <v/>
+      </c>
+      <c r="E17" s="61">
+        <f>'Data'!F26*1000000</f>
+        <v/>
+      </c>
+      <c r="F17" s="61">
+        <f>'Data'!F27*1000000</f>
+        <v/>
+      </c>
+      <c r="G17" s="61">
+        <f>'Data'!F28*1000000</f>
+        <v/>
+      </c>
+      <c r="H17" s="61">
+        <f>'Data'!F29*1000000</f>
+        <v/>
+      </c>
+      <c r="I17" s="62">
+        <f>IFERROR((D17/G17)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="62">
+        <f>IFERROR((E17/H17)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="62">
+        <f>IFERROR((F17/H17)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="62">
+        <f>IFERROR(I17+J17-K17,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2020</v>
+      </c>
+      <c r="D18" s="61">
+        <f>'Data'!G25*1000000</f>
+        <v/>
+      </c>
+      <c r="E18" s="61">
+        <f>'Data'!G26*1000000</f>
+        <v/>
+      </c>
+      <c r="F18" s="61">
+        <f>'Data'!G27*1000000</f>
+        <v/>
+      </c>
+      <c r="G18" s="61">
+        <f>'Data'!G28*1000000</f>
+        <v/>
+      </c>
+      <c r="H18" s="61">
+        <f>'Data'!G29*1000000</f>
+        <v/>
+      </c>
+      <c r="I18" s="62">
+        <f>IFERROR((D18/G18)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="62">
+        <f>IFERROR((E18/H18)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="62">
+        <f>IFERROR((F18/H18)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="62">
+        <f>IFERROR(I18+J18-K18,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Walmart Inc.</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2021</v>
+      </c>
+      <c r="D19" s="61">
+        <f>'Data'!H25*1000000</f>
+        <v/>
+      </c>
+      <c r="E19" s="61">
+        <f>'Data'!H26*1000000</f>
+        <v/>
+      </c>
+      <c r="F19" s="61">
+        <f>'Data'!H27*1000000</f>
+        <v/>
+      </c>
+      <c r="G19" s="61">
+        <f>'Data'!H28*1000000</f>
+        <v/>
+      </c>
+      <c r="H19" s="61">
+        <f>'Data'!H29*1000000</f>
+        <v/>
+      </c>
+      <c r="I19" s="62">
+        <f>IFERROR((D19/G19)*365,"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="62">
+        <f>IFERROR((E19/H19)*365,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="62">
+        <f>IFERROR((F19/H19)*365,"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="62">
+        <f>IFERROR(I19+J19-K19,"")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>